<commit_message>
Add facilities tracking section for dept6
</commit_message>
<xml_diff>
--- a/المستخدمين.xlsx
+++ b/المستخدمين.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\تطبيقي\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022AC262-49E9-4CF6-9109-293B1841BC51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FAA3ED2-2393-4E14-B447-AD5C4678ACDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8C11EB78-F252-4332-9410-1458DD7567FE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>training@gahar.gov.eg</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>abdullahbido@gmail.com</t>
+  </si>
+  <si>
+    <t>admin@gahar.gov.eg</t>
   </si>
 </sst>
 </file>
@@ -478,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B05737-2DBB-47FB-ADE8-231989853B7E}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.77734375" customWidth="1"/>
@@ -560,6 +563,14 @@
         <v>18</v>
       </c>
     </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{3802534C-3D19-462A-8158-A3A5413FCEFD}"/>
@@ -568,6 +579,7 @@
     <hyperlink ref="A5" r:id="rId4" xr:uid="{F6C0A7DF-74A7-45A7-809D-72A0083AFA29}"/>
     <hyperlink ref="A6" r:id="rId5" xr:uid="{E37180EF-F6F9-440B-82B5-A470D304F69D}"/>
     <hyperlink ref="A7" r:id="rId6" xr:uid="{EB0EAFB2-4D1E-49EB-8B2C-0C27390C368F}"/>
+    <hyperlink ref="A8" r:id="rId7" xr:uid="{F7A1EDBF-8DDD-48D8-8793-B30D50DD50BD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update dashboards and admin audit governing authority field
</commit_message>
<xml_diff>
--- a/المستخدمين.xlsx
+++ b/المستخدمين.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\تطبيقي\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D22977-D5C0-4792-8504-EDA8442C2AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B1AA06A-D0DE-4662-8E87-19C7796C7901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8C11EB78-F252-4332-9410-1458DD7567FE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>training@gahar.gov.eg</t>
   </si>
@@ -153,6 +153,15 @@
   </si>
   <si>
     <t>RevGahar_2026</t>
+  </si>
+  <si>
+    <t>أماني المعداوي</t>
+  </si>
+  <si>
+    <t>Amany_2026</t>
+  </si>
+  <si>
+    <t>amany@gahar.gov.eg</t>
   </si>
 </sst>
 </file>
@@ -535,7 +544,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B05737-2DBB-47FB-ADE8-231989853B7E}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.77734375" customWidth="1"/>
@@ -689,6 +698,17 @@
       </c>
       <c r="C14" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -709,6 +729,7 @@
     <hyperlink ref="A13" r:id="rId14" xr:uid="{1E309800-E1D7-4E32-B3AB-1033D20D12E2}"/>
     <hyperlink ref="B13" r:id="rId15" xr:uid="{B65A6043-234D-4401-B3F1-D04C2996AFF7}"/>
     <hyperlink ref="A14" r:id="rId16" xr:uid="{AF761C99-AC62-49B5-9FD5-10D8988BA526}"/>
+    <hyperlink ref="A15" r:id="rId17" xr:uid="{55569F02-F190-4B1B-96CD-0CE82C04A630}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Security: Remove hardcoded admin credentials from auth.ts
</commit_message>
<xml_diff>
--- a/المستخدمين.xlsx
+++ b/المستخدمين.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\تطبيقي\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B1AA06A-D0DE-4662-8E87-19C7796C7901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1E0870-60B2-44B4-A0C6-E7557CD22419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8C11EB78-F252-4332-9410-1458DD7567FE}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>Tr1234</t>
   </si>
   <si>
-    <t>standards@gahar.gov.eg</t>
-  </si>
-  <si>
     <t>St1234</t>
   </si>
   <si>
@@ -162,6 +159,9 @@
   </si>
   <si>
     <t>amany@gahar.gov.eg</t>
+  </si>
+  <si>
+    <t>standard@gahar.gov.eg</t>
   </si>
 </sst>
 </file>
@@ -554,13 +554,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>10</v>
-      </c>
-      <c r="C1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -571,144 +571,144 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
         <v>20</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
         <v>23</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
         <v>26</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" t="s">
         <v>34</v>
-      </c>
-      <c r="C13" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" t="s">
         <v>37</v>
       </c>
-      <c r="B14" t="s">
-        <v>38</v>
-      </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>